<commit_message>
Updated the workflow progress
</commit_message>
<xml_diff>
--- a/Internal-Security_Framework_7Week_Gantt_Chart.xlsx
+++ b/Internal-Security_Framework_7Week_Gantt_Chart.xlsx
@@ -343,7 +343,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -372,6 +372,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAFD095"/>
+        <bgColor rgb="FFCBD5E1"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,152 +478,160 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -646,7 +660,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF0D9488"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF9333EA"/>
@@ -876,118 +890,118 @@
   <dimension ref="A1:I41"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="5" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="9"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
       <c r="F8" s="15"/>
@@ -1002,19 +1016,19 @@
       <c r="B9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="9"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="18"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="15"/>
@@ -1026,25 +1040,25 @@
       <c r="I10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="12"/>
+      <c r="C11" s="13"/>
       <c r="D11" s="18"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="15"/>
@@ -1062,19 +1076,19 @@
       <c r="B13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
       <c r="E13" s="21"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="15"/>
@@ -1086,25 +1100,25 @@
       <c r="I14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
       <c r="E15" s="21"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="23" t="s">
         <v>33</v>
       </c>
       <c r="C16" s="15"/>
@@ -1116,145 +1130,145 @@
       <c r="I16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="23" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
-      <c r="F18" s="24"/>
+      <c r="F18" s="26"/>
       <c r="G18" s="15"/>
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="23" t="s">
         <v>41</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="24"/>
+      <c r="F20" s="26"/>
       <c r="G20" s="15"/>
       <c r="H20" s="15"/>
       <c r="I20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="23" t="s">
         <v>45</v>
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
-      <c r="G22" s="27"/>
+      <c r="G22" s="29"/>
       <c r="H22" s="15"/>
       <c r="I22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
       <c r="E24" s="15"/>
       <c r="F24" s="15"/>
-      <c r="G24" s="27"/>
+      <c r="G24" s="29"/>
       <c r="H24" s="15"/>
       <c r="I24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="9"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C26" s="15"/>
@@ -1262,29 +1276,29 @@
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="30"/>
+      <c r="H26" s="32"/>
       <c r="I26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="12"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="23" t="s">
         <v>57</v>
       </c>
       <c r="C28" s="15"/>
@@ -1292,29 +1306,29 @@
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="30"/>
+      <c r="H28" s="32"/>
       <c r="I28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31" t="s">
+      <c r="A29" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="33"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="35"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="23" t="s">
         <v>61</v>
       </c>
       <c r="C30" s="15"/>
@@ -1323,28 +1337,28 @@
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
       <c r="H30" s="15"/>
-      <c r="I30" s="33"/>
+      <c r="I30" s="35"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="33"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="35"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="23" t="s">
         <v>65</v>
       </c>
       <c r="C32" s="15"/>
@@ -1353,125 +1367,125 @@
       <c r="F32" s="15"/>
       <c r="G32" s="15"/>
       <c r="H32" s="15"/>
-      <c r="I32" s="33"/>
+      <c r="I32" s="35"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="34"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="36"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="35" t="s">
+      <c r="A35" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="B35" s="36" t="s">
+      <c r="B35" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="35" t="s">
+      <c r="A36" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="36" t="s">
+      <c r="B36" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="35" t="s">
+      <c r="A37" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="36" t="s">
+      <c r="B37" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="35" t="s">
+      <c r="A38" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="36" t="s">
+      <c r="B38" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="36" t="s">
+      <c r="B39" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="35" t="s">
+      <c r="A40" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="36" t="s">
+      <c r="B40" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="35" t="s">
+      <c r="A41" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="36" t="s">
+      <c r="B41" s="38" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>